<commit_message>
make a url for every site
</commit_message>
<xml_diff>
--- a/public/gny committee mapping.xlsx
+++ b/public/gny committee mapping.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\committees list app\committees-mapping\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32AB6529-684F-4998-9858-070FCBB893DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8931210B-59E6-4775-A452-0810261C9F1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9EEC2C38-FF41-4F97-B0EC-E60FF86960E5}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9EEC2C38-FF41-4F97-B0EC-E60FF86960E5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$E$312</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$E$438</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -2072,16 +2072,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F478A83-309B-482A-B8B0-EA389326FD99}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:E438"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="18.7109375" customWidth="1"/>
+    <col min="1" max="2" width="18.6640625" customWidth="1"/>
     <col min="3" max="3" width="44" customWidth="1"/>
-    <col min="4" max="4" width="35.7109375" customWidth="1"/>
-    <col min="5" max="5" width="12.140625" customWidth="1"/>
+    <col min="4" max="4" width="35.6640625" customWidth="1"/>
+    <col min="5" max="5" width="12.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>521</v>
       </c>
@@ -2098,7 +2099,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>522</v>
       </c>
@@ -2115,7 +2116,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>522</v>
       </c>
@@ -2132,7 +2133,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>522</v>
       </c>
@@ -2149,7 +2150,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>522</v>
       </c>
@@ -2166,7 +2167,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>522</v>
       </c>
@@ -2183,7 +2184,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>522</v>
       </c>
@@ -2200,7 +2201,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>522</v>
       </c>
@@ -2217,7 +2218,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>522</v>
       </c>
@@ -2234,7 +2235,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>522</v>
       </c>
@@ -2251,7 +2252,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>522</v>
       </c>
@@ -2268,7 +2269,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>522</v>
       </c>
@@ -2285,7 +2286,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>522</v>
       </c>
@@ -2302,7 +2303,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>522</v>
       </c>
@@ -2319,7 +2320,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>522</v>
       </c>
@@ -2336,7 +2337,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>522</v>
       </c>
@@ -2353,7 +2354,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>522</v>
       </c>
@@ -2370,7 +2371,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>522</v>
       </c>
@@ -2387,7 +2388,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>522</v>
       </c>
@@ -2404,7 +2405,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>522</v>
       </c>
@@ -2421,7 +2422,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>522</v>
       </c>
@@ -2438,7 +2439,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>522</v>
       </c>
@@ -2455,7 +2456,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>522</v>
       </c>
@@ -2472,7 +2473,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>522</v>
       </c>
@@ -2489,7 +2490,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>522</v>
       </c>
@@ -2506,7 +2507,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>522</v>
       </c>
@@ -2523,7 +2524,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>522</v>
       </c>
@@ -2540,7 +2541,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>522</v>
       </c>
@@ -2557,7 +2558,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>522</v>
       </c>
@@ -2574,7 +2575,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>522</v>
       </c>
@@ -2591,7 +2592,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>522</v>
       </c>
@@ -2608,7 +2609,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>522</v>
       </c>
@@ -2625,7 +2626,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>522</v>
       </c>
@@ -2642,7 +2643,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>522</v>
       </c>
@@ -2659,7 +2660,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>522</v>
       </c>
@@ -2676,7 +2677,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>522</v>
       </c>
@@ -2693,7 +2694,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>522</v>
       </c>
@@ -2710,7 +2711,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>522</v>
       </c>
@@ -2727,7 +2728,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>522</v>
       </c>
@@ -2744,7 +2745,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>522</v>
       </c>
@@ -2761,7 +2762,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>522</v>
       </c>
@@ -2778,7 +2779,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>522</v>
       </c>
@@ -2795,7 +2796,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>522</v>
       </c>
@@ -2812,7 +2813,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>522</v>
       </c>
@@ -2829,7 +2830,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>522</v>
       </c>
@@ -2846,7 +2847,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>522</v>
       </c>
@@ -2863,7 +2864,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>522</v>
       </c>
@@ -2880,7 +2881,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>522</v>
       </c>
@@ -2897,7 +2898,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>522</v>
       </c>
@@ -2914,7 +2915,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>522</v>
       </c>
@@ -2931,7 +2932,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>522</v>
       </c>
@@ -2948,7 +2949,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>522</v>
       </c>
@@ -2965,7 +2966,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>522</v>
       </c>
@@ -2982,7 +2983,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>522</v>
       </c>
@@ -2999,7 +3000,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>522</v>
       </c>
@@ -3016,7 +3017,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>522</v>
       </c>
@@ -3033,7 +3034,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>522</v>
       </c>
@@ -3050,7 +3051,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>522</v>
       </c>
@@ -3067,7 +3068,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>522</v>
       </c>
@@ -3084,7 +3085,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>522</v>
       </c>
@@ -3101,7 +3102,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>522</v>
       </c>
@@ -3118,7 +3119,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>522</v>
       </c>
@@ -3135,7 +3136,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>522</v>
       </c>
@@ -3152,7 +3153,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>522</v>
       </c>
@@ -3169,7 +3170,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>522</v>
       </c>
@@ -3186,7 +3187,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>522</v>
       </c>
@@ -3203,7 +3204,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>522</v>
       </c>
@@ -3220,7 +3221,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>522</v>
       </c>
@@ -3237,7 +3238,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>522</v>
       </c>
@@ -3254,7 +3255,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>522</v>
       </c>
@@ -3271,7 +3272,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>522</v>
       </c>
@@ -3288,7 +3289,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>522</v>
       </c>
@@ -3305,7 +3306,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>522</v>
       </c>
@@ -3322,7 +3323,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>522</v>
       </c>
@@ -3339,7 +3340,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>522</v>
       </c>
@@ -3356,7 +3357,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>522</v>
       </c>
@@ -3373,7 +3374,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>522</v>
       </c>
@@ -3390,7 +3391,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>522</v>
       </c>
@@ -3407,7 +3408,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>522</v>
       </c>
@@ -3424,7 +3425,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>522</v>
       </c>
@@ -3441,7 +3442,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>522</v>
       </c>
@@ -3458,7 +3459,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>522</v>
       </c>
@@ -3475,7 +3476,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>522</v>
       </c>
@@ -3492,7 +3493,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>522</v>
       </c>
@@ -3509,7 +3510,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>522</v>
       </c>
@@ -3526,7 +3527,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>522</v>
       </c>
@@ -3543,7 +3544,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>522</v>
       </c>
@@ -3560,7 +3561,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>522</v>
       </c>
@@ -3577,7 +3578,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>522</v>
       </c>
@@ -3594,7 +3595,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>522</v>
       </c>
@@ -3611,7 +3612,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>522</v>
       </c>
@@ -3628,7 +3629,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>522</v>
       </c>
@@ -3645,7 +3646,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>522</v>
       </c>
@@ -3662,7 +3663,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>522</v>
       </c>
@@ -3679,7 +3680,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>522</v>
       </c>
@@ -3696,7 +3697,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>522</v>
       </c>
@@ -3713,7 +3714,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>522</v>
       </c>
@@ -3730,7 +3731,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>522</v>
       </c>
@@ -3747,7 +3748,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>522</v>
       </c>
@@ -3764,7 +3765,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>522</v>
       </c>
@@ -3781,7 +3782,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>522</v>
       </c>
@@ -3798,7 +3799,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>522</v>
       </c>
@@ -3815,7 +3816,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>522</v>
       </c>
@@ -3832,7 +3833,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>522</v>
       </c>
@@ -3849,7 +3850,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>522</v>
       </c>
@@ -3866,7 +3867,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>522</v>
       </c>
@@ -3883,7 +3884,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>522</v>
       </c>
@@ -3900,7 +3901,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>522</v>
       </c>
@@ -3917,7 +3918,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>522</v>
       </c>
@@ -3934,7 +3935,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>522</v>
       </c>
@@ -3951,7 +3952,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>522</v>
       </c>
@@ -3968,7 +3969,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>522</v>
       </c>
@@ -3985,7 +3986,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>522</v>
       </c>
@@ -4002,7 +4003,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>522</v>
       </c>
@@ -4019,7 +4020,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>522</v>
       </c>
@@ -4036,7 +4037,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>522</v>
       </c>
@@ -4053,7 +4054,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>522</v>
       </c>
@@ -4070,7 +4071,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>522</v>
       </c>
@@ -4087,7 +4088,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>522</v>
       </c>
@@ -4104,7 +4105,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>522</v>
       </c>
@@ -4121,7 +4122,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>522</v>
       </c>
@@ -4138,7 +4139,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>522</v>
       </c>
@@ -4155,7 +4156,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>522</v>
       </c>
@@ -4172,7 +4173,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>522</v>
       </c>
@@ -4189,7 +4190,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>522</v>
       </c>
@@ -4206,7 +4207,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>522</v>
       </c>
@@ -4223,7 +4224,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>522</v>
       </c>
@@ -4240,7 +4241,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>522</v>
       </c>
@@ -4257,7 +4258,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>522</v>
       </c>
@@ -4274,7 +4275,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>522</v>
       </c>
@@ -4291,7 +4292,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>522</v>
       </c>
@@ -4308,7 +4309,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>522</v>
       </c>
@@ -4325,7 +4326,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>522</v>
       </c>
@@ -4342,7 +4343,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>522</v>
       </c>
@@ -4359,7 +4360,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>522</v>
       </c>
@@ -4376,7 +4377,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>522</v>
       </c>
@@ -4393,7 +4394,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>522</v>
       </c>
@@ -4410,7 +4411,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>522</v>
       </c>
@@ -4427,7 +4428,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>522</v>
       </c>
@@ -4444,7 +4445,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>522</v>
       </c>
@@ -4461,7 +4462,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>522</v>
       </c>
@@ -4478,7 +4479,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>522</v>
       </c>
@@ -4495,7 +4496,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>522</v>
       </c>
@@ -4512,7 +4513,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>522</v>
       </c>
@@ -4529,7 +4530,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>522</v>
       </c>
@@ -4546,7 +4547,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>522</v>
       </c>
@@ -4563,7 +4564,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>522</v>
       </c>
@@ -4580,7 +4581,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>522</v>
       </c>
@@ -4597,7 +4598,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>522</v>
       </c>
@@ -4614,7 +4615,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>522</v>
       </c>
@@ -4631,7 +4632,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>522</v>
       </c>
@@ -4648,7 +4649,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>522</v>
       </c>
@@ -4665,7 +4666,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>522</v>
       </c>
@@ -4682,7 +4683,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>522</v>
       </c>
@@ -4699,7 +4700,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
         <v>522</v>
       </c>
@@ -4716,7 +4717,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>522</v>
       </c>
@@ -4733,7 +4734,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>522</v>
       </c>
@@ -4750,7 +4751,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>522</v>
       </c>
@@ -4767,7 +4768,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>522</v>
       </c>
@@ -4784,7 +4785,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>522</v>
       </c>
@@ -4801,7 +4802,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>522</v>
       </c>
@@ -4818,7 +4819,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>522</v>
       </c>
@@ -4835,7 +4836,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>522</v>
       </c>
@@ -4852,7 +4853,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>522</v>
       </c>
@@ -4869,7 +4870,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
         <v>522</v>
       </c>
@@ -4886,7 +4887,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
         <v>522</v>
       </c>
@@ -4903,7 +4904,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>522</v>
       </c>
@@ -4920,7 +4921,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>522</v>
       </c>
@@ -4937,7 +4938,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>522</v>
       </c>
@@ -4954,7 +4955,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>522</v>
       </c>
@@ -4971,7 +4972,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
         <v>522</v>
       </c>
@@ -4988,7 +4989,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
         <v>522</v>
       </c>
@@ -5005,7 +5006,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
         <v>522</v>
       </c>
@@ -5022,7 +5023,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
         <v>522</v>
       </c>
@@ -5039,7 +5040,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
         <v>522</v>
       </c>
@@ -5056,7 +5057,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
         <v>522</v>
       </c>
@@ -5073,7 +5074,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
         <v>522</v>
       </c>
@@ -5090,7 +5091,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A178" t="s">
         <v>522</v>
       </c>
@@ -5107,7 +5108,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
         <v>522</v>
       </c>
@@ -5124,7 +5125,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
         <v>522</v>
       </c>
@@ -5141,7 +5142,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
         <v>522</v>
       </c>
@@ -5158,7 +5159,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A182" t="s">
         <v>522</v>
       </c>
@@ -5175,7 +5176,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A183" t="s">
         <v>522</v>
       </c>
@@ -5192,7 +5193,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A184" t="s">
         <v>522</v>
       </c>
@@ -5209,7 +5210,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A185" t="s">
         <v>522</v>
       </c>
@@ -5226,7 +5227,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A186" t="s">
         <v>522</v>
       </c>
@@ -5243,7 +5244,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
         <v>522</v>
       </c>
@@ -5260,7 +5261,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A188" t="s">
         <v>522</v>
       </c>
@@ -5277,7 +5278,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
         <v>522</v>
       </c>
@@ -5294,7 +5295,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
         <v>522</v>
       </c>
@@ -5311,7 +5312,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A191" t="s">
         <v>522</v>
       </c>
@@ -5328,7 +5329,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A192" t="s">
         <v>523</v>
       </c>
@@ -5345,7 +5346,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A193" t="s">
         <v>523</v>
       </c>
@@ -5362,7 +5363,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A194" t="s">
         <v>523</v>
       </c>
@@ -5379,7 +5380,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A195" t="s">
         <v>523</v>
       </c>
@@ -5396,7 +5397,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A196" t="s">
         <v>523</v>
       </c>
@@ -5413,7 +5414,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
         <v>523</v>
       </c>
@@ -5430,7 +5431,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A198" t="s">
         <v>523</v>
       </c>
@@ -5447,7 +5448,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A199" t="s">
         <v>523</v>
       </c>
@@ -5464,7 +5465,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A200" t="s">
         <v>523</v>
       </c>
@@ -5481,7 +5482,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A201" t="s">
         <v>523</v>
       </c>
@@ -5498,7 +5499,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A202" t="s">
         <v>523</v>
       </c>
@@ -5515,7 +5516,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A203" t="s">
         <v>523</v>
       </c>
@@ -5532,7 +5533,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A204" t="s">
         <v>523</v>
       </c>
@@ -5549,7 +5550,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A205" t="s">
         <v>523</v>
       </c>
@@ -5566,7 +5567,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A206" t="s">
         <v>523</v>
       </c>
@@ -5583,7 +5584,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A207" t="s">
         <v>523</v>
       </c>
@@ -5600,7 +5601,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="208" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A208" t="s">
         <v>523</v>
       </c>
@@ -5617,7 +5618,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="209" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A209" t="s">
         <v>523</v>
       </c>
@@ -5634,7 +5635,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="210" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A210" t="s">
         <v>523</v>
       </c>
@@ -5651,7 +5652,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="211" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A211" t="s">
         <v>523</v>
       </c>
@@ -5668,7 +5669,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="212" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A212" t="s">
         <v>523</v>
       </c>
@@ -5685,7 +5686,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="213" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A213" t="s">
         <v>523</v>
       </c>
@@ -5702,7 +5703,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="214" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A214" t="s">
         <v>523</v>
       </c>
@@ -5719,7 +5720,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="215" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A215" t="s">
         <v>523</v>
       </c>
@@ -5736,7 +5737,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="216" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A216" t="s">
         <v>523</v>
       </c>
@@ -5753,7 +5754,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="217" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A217" t="s">
         <v>523</v>
       </c>
@@ -5770,7 +5771,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="218" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A218" t="s">
         <v>523</v>
       </c>
@@ -5787,7 +5788,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="219" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A219" t="s">
         <v>523</v>
       </c>
@@ -5804,7 +5805,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="220" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A220" t="s">
         <v>523</v>
       </c>
@@ -5821,7 +5822,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="221" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A221" t="s">
         <v>523</v>
       </c>
@@ -5838,7 +5839,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="222" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A222" t="s">
         <v>523</v>
       </c>
@@ -5855,7 +5856,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="223" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A223" t="s">
         <v>523</v>
       </c>
@@ -5872,7 +5873,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="224" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A224" t="s">
         <v>523</v>
       </c>
@@ -5889,7 +5890,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="225" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A225" t="s">
         <v>523</v>
       </c>
@@ -5906,7 +5907,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="226" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A226" t="s">
         <v>523</v>
       </c>
@@ -5923,7 +5924,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="227" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A227" t="s">
         <v>523</v>
       </c>
@@ -5940,7 +5941,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="228" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A228" t="s">
         <v>523</v>
       </c>
@@ -5957,7 +5958,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="229" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A229" t="s">
         <v>523</v>
       </c>
@@ -5974,7 +5975,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="230" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A230" t="s">
         <v>523</v>
       </c>
@@ -5991,7 +5992,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="231" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A231" t="s">
         <v>523</v>
       </c>
@@ -6008,7 +6009,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="232" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A232" t="s">
         <v>523</v>
       </c>
@@ -6025,7 +6026,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="233" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A233" t="s">
         <v>523</v>
       </c>
@@ -6042,7 +6043,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="234" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A234" t="s">
         <v>523</v>
       </c>
@@ -6059,7 +6060,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="235" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A235" t="s">
         <v>523</v>
       </c>
@@ -6076,7 +6077,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="236" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A236" t="s">
         <v>523</v>
       </c>
@@ -6093,7 +6094,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="237" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A237" t="s">
         <v>523</v>
       </c>
@@ -6110,7 +6111,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="238" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A238" t="s">
         <v>523</v>
       </c>
@@ -6127,7 +6128,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="239" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A239" t="s">
         <v>523</v>
       </c>
@@ -6144,7 +6145,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="240" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A240" t="s">
         <v>523</v>
       </c>
@@ -6161,7 +6162,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="241" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A241" t="s">
         <v>523</v>
       </c>
@@ -6178,7 +6179,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="242" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A242" t="s">
         <v>523</v>
       </c>
@@ -6195,7 +6196,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="243" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A243" t="s">
         <v>523</v>
       </c>
@@ -6212,7 +6213,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="244" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A244" t="s">
         <v>523</v>
       </c>
@@ -6229,7 +6230,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="245" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A245" t="s">
         <v>523</v>
       </c>
@@ -6246,7 +6247,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="246" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A246" t="s">
         <v>523</v>
       </c>
@@ -6263,7 +6264,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="247" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A247" t="s">
         <v>523</v>
       </c>
@@ -6280,7 +6281,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="248" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A248" t="s">
         <v>523</v>
       </c>
@@ -6297,7 +6298,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="249" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A249" t="s">
         <v>523</v>
       </c>
@@ -6314,7 +6315,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="250" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A250" t="s">
         <v>523</v>
       </c>
@@ -6331,7 +6332,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="251" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A251" t="s">
         <v>523</v>
       </c>
@@ -6348,7 +6349,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="252" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A252" t="s">
         <v>523</v>
       </c>
@@ -6365,7 +6366,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="253" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A253" t="s">
         <v>523</v>
       </c>
@@ -6382,7 +6383,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="254" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A254" t="s">
         <v>523</v>
       </c>
@@ -6399,7 +6400,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="255" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A255" t="s">
         <v>523</v>
       </c>
@@ -6416,7 +6417,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="256" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A256" t="s">
         <v>523</v>
       </c>
@@ -6433,7 +6434,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="257" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A257" t="s">
         <v>523</v>
       </c>
@@ -6450,7 +6451,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="258" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A258" t="s">
         <v>523</v>
       </c>
@@ -6467,7 +6468,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="259" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A259" t="s">
         <v>523</v>
       </c>
@@ -6484,7 +6485,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="260" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A260" t="s">
         <v>523</v>
       </c>
@@ -6501,7 +6502,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="261" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A261" t="s">
         <v>523</v>
       </c>
@@ -6518,7 +6519,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="262" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A262" t="s">
         <v>523</v>
       </c>
@@ -6535,7 +6536,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="263" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A263" t="s">
         <v>523</v>
       </c>
@@ -6552,7 +6553,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="264" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A264" t="s">
         <v>523</v>
       </c>
@@ -6569,7 +6570,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="265" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A265" t="s">
         <v>523</v>
       </c>
@@ -6586,7 +6587,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="266" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A266" t="s">
         <v>523</v>
       </c>
@@ -6603,7 +6604,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="267" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A267" t="s">
         <v>523</v>
       </c>
@@ -6620,7 +6621,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="268" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A268" t="s">
         <v>523</v>
       </c>
@@ -6637,7 +6638,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="269" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A269" t="s">
         <v>523</v>
       </c>
@@ -6654,7 +6655,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="270" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A270" t="s">
         <v>523</v>
       </c>
@@ -6671,7 +6672,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="271" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A271" t="s">
         <v>523</v>
       </c>
@@ -6688,7 +6689,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="272" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A272" t="s">
         <v>523</v>
       </c>
@@ -6705,7 +6706,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="273" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A273" t="s">
         <v>523</v>
       </c>
@@ -6722,7 +6723,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="274" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A274" t="s">
         <v>523</v>
       </c>
@@ -6739,7 +6740,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="275" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A275" t="s">
         <v>523</v>
       </c>
@@ -6756,7 +6757,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="276" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A276" t="s">
         <v>523</v>
       </c>
@@ -6773,7 +6774,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="277" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A277" t="s">
         <v>523</v>
       </c>
@@ -6790,7 +6791,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="278" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A278" t="s">
         <v>523</v>
       </c>
@@ -6807,7 +6808,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="279" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A279" t="s">
         <v>523</v>
       </c>
@@ -6824,7 +6825,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="280" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A280" t="s">
         <v>523</v>
       </c>
@@ -6841,7 +6842,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="281" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A281" t="s">
         <v>523</v>
       </c>
@@ -6858,7 +6859,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="282" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A282" t="s">
         <v>523</v>
       </c>
@@ -6875,7 +6876,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="283" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A283" t="s">
         <v>523</v>
       </c>
@@ -6892,7 +6893,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="284" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A284" t="s">
         <v>523</v>
       </c>
@@ -6909,7 +6910,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="285" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A285" t="s">
         <v>523</v>
       </c>
@@ -6926,7 +6927,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="286" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A286" t="s">
         <v>523</v>
       </c>
@@ -6943,7 +6944,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="287" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A287" t="s">
         <v>523</v>
       </c>
@@ -6960,7 +6961,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="288" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A288" t="s">
         <v>523</v>
       </c>
@@ -6977,7 +6978,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="289" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A289" t="s">
         <v>523</v>
       </c>
@@ -6994,7 +6995,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="290" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A290" t="s">
         <v>523</v>
       </c>
@@ -7011,7 +7012,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="291" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A291" t="s">
         <v>523</v>
       </c>
@@ -7028,7 +7029,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="292" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A292" t="s">
         <v>523</v>
       </c>
@@ -7045,7 +7046,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="293" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A293" t="s">
         <v>523</v>
       </c>
@@ -7062,7 +7063,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="294" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A294" t="s">
         <v>523</v>
       </c>
@@ -7079,7 +7080,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="295" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A295" t="s">
         <v>523</v>
       </c>
@@ -7096,7 +7097,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="296" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A296" t="s">
         <v>523</v>
       </c>
@@ -7113,7 +7114,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="297" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A297" t="s">
         <v>523</v>
       </c>
@@ -7130,7 +7131,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="298" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A298" t="s">
         <v>523</v>
       </c>
@@ -7147,7 +7148,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="299" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A299" t="s">
         <v>522</v>
       </c>
@@ -7161,7 +7162,7 @@
         <v>524</v>
       </c>
     </row>
-    <row r="300" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A300" t="s">
         <v>522</v>
       </c>
@@ -7175,7 +7176,7 @@
         <v>525</v>
       </c>
     </row>
-    <row r="301" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A301" t="s">
         <v>522</v>
       </c>
@@ -7189,7 +7190,7 @@
         <v>526</v>
       </c>
     </row>
-    <row r="302" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A302" t="s">
         <v>522</v>
       </c>
@@ -7203,7 +7204,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="303" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A303" t="s">
         <v>522</v>
       </c>
@@ -7217,7 +7218,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="304" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A304" t="s">
         <v>522</v>
       </c>
@@ -7231,7 +7232,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="305" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A305" t="s">
         <v>522</v>
       </c>
@@ -7245,7 +7246,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="306" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A306" t="s">
         <v>522</v>
       </c>
@@ -7259,7 +7260,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="307" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A307" t="s">
         <v>522</v>
       </c>
@@ -7273,7 +7274,7 @@
         <v>533</v>
       </c>
     </row>
-    <row r="308" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A308" t="s">
         <v>522</v>
       </c>
@@ -7287,7 +7288,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="309" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A309" t="s">
         <v>522</v>
       </c>
@@ -7301,7 +7302,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="310" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A310" t="s">
         <v>522</v>
       </c>
@@ -7315,7 +7316,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="311" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A311" t="s">
         <v>522</v>
       </c>
@@ -7329,7 +7330,7 @@
         <v>537</v>
       </c>
     </row>
-    <row r="312" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A312" t="s">
         <v>522</v>
       </c>
@@ -7343,7 +7344,7 @@
         <v>538</v>
       </c>
     </row>
-    <row r="313" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A313" t="s">
         <v>523</v>
       </c>
@@ -7357,7 +7358,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="314" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A314" t="s">
         <v>523</v>
       </c>
@@ -7371,7 +7372,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="315" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A315" t="s">
         <v>523</v>
       </c>
@@ -7385,7 +7386,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="316" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A316" t="s">
         <v>523</v>
       </c>
@@ -7399,7 +7400,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="317" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A317" t="s">
         <v>523</v>
       </c>
@@ -7413,7 +7414,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="318" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A318" t="s">
         <v>523</v>
       </c>
@@ -7427,7 +7428,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="319" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A319" t="s">
         <v>523</v>
       </c>
@@ -7441,7 +7442,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="320" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A320" t="s">
         <v>523</v>
       </c>
@@ -7455,7 +7456,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="321" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A321" t="s">
         <v>523</v>
       </c>
@@ -7469,7 +7470,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="322" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A322" t="s">
         <v>523</v>
       </c>
@@ -7483,7 +7484,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="323" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A323" t="s">
         <v>523</v>
       </c>
@@ -7497,7 +7498,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="324" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A324" t="s">
         <v>523</v>
       </c>
@@ -7511,7 +7512,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="325" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A325" t="s">
         <v>523</v>
       </c>
@@ -7525,7 +7526,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="326" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A326" t="s">
         <v>523</v>
       </c>
@@ -7539,7 +7540,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="327" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A327" t="s">
         <v>523</v>
       </c>
@@ -7553,7 +7554,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="328" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A328" t="s">
         <v>523</v>
       </c>
@@ -7567,7 +7568,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="329" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A329" t="s">
         <v>523</v>
       </c>
@@ -7581,7 +7582,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="330" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A330" t="s">
         <v>523</v>
       </c>
@@ -7595,7 +7596,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="331" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A331" t="s">
         <v>523</v>
       </c>
@@ -7609,7 +7610,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="332" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A332" t="s">
         <v>523</v>
       </c>
@@ -7623,7 +7624,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="333" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A333" t="s">
         <v>523</v>
       </c>
@@ -7637,7 +7638,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="334" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A334" t="s">
         <v>523</v>
       </c>
@@ -7651,7 +7652,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="335" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A335" t="s">
         <v>523</v>
       </c>
@@ -7665,7 +7666,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="336" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A336" t="s">
         <v>523</v>
       </c>
@@ -7679,7 +7680,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="337" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A337" t="s">
         <v>523</v>
       </c>
@@ -7693,7 +7694,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="338" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A338" t="s">
         <v>523</v>
       </c>
@@ -7707,7 +7708,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="339" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A339" t="s">
         <v>523</v>
       </c>
@@ -7721,7 +7722,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="340" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A340" t="s">
         <v>523</v>
       </c>
@@ -7735,7 +7736,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="341" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A341" t="s">
         <v>523</v>
       </c>
@@ -7749,7 +7750,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="342" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A342" t="s">
         <v>523</v>
       </c>
@@ -7763,7 +7764,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="343" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A343" t="s">
         <v>523</v>
       </c>
@@ -7777,7 +7778,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="344" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A344" t="s">
         <v>523</v>
       </c>
@@ -7791,7 +7792,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="345" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="345" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A345" t="s">
         <v>523</v>
       </c>
@@ -7805,7 +7806,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="346" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="346" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A346" t="s">
         <v>523</v>
       </c>
@@ -7819,7 +7820,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="347" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="347" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A347" t="s">
         <v>523</v>
       </c>
@@ -7833,7 +7834,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="348" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="348" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A348" t="s">
         <v>523</v>
       </c>
@@ -7847,7 +7848,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="349" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="349" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A349" t="s">
         <v>523</v>
       </c>
@@ -7861,7 +7862,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="350" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="350" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A350" t="s">
         <v>523</v>
       </c>
@@ -7875,7 +7876,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="351" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="351" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A351" t="s">
         <v>523</v>
       </c>
@@ -7889,7 +7890,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="352" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="352" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A352" t="s">
         <v>523</v>
       </c>
@@ -7903,7 +7904,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="353" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="353" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A353" t="s">
         <v>523</v>
       </c>
@@ -7917,7 +7918,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="354" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="354" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A354" t="s">
         <v>523</v>
       </c>
@@ -7931,7 +7932,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="355" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="355" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A355" t="s">
         <v>523</v>
       </c>
@@ -7945,7 +7946,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="356" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="356" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A356" t="s">
         <v>523</v>
       </c>
@@ -7959,7 +7960,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="357" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="357" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A357" t="s">
         <v>523</v>
       </c>
@@ -7973,7 +7974,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="358" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="358" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A358" t="s">
         <v>523</v>
       </c>
@@ -7987,7 +7988,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="359" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="359" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A359" t="s">
         <v>523</v>
       </c>
@@ -8001,7 +8002,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="360" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="360" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A360" t="s">
         <v>523</v>
       </c>
@@ -8015,7 +8016,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="361" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="361" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A361" t="s">
         <v>523</v>
       </c>
@@ -8029,7 +8030,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="362" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="362" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A362" t="s">
         <v>523</v>
       </c>
@@ -8043,7 +8044,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="363" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="363" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A363" t="s">
         <v>523</v>
       </c>
@@ -8057,7 +8058,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="364" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="364" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A364" t="s">
         <v>523</v>
       </c>
@@ -8071,7 +8072,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="365" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="365" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A365" t="s">
         <v>523</v>
       </c>
@@ -8085,7 +8086,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="366" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="366" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A366" t="s">
         <v>523</v>
       </c>
@@ -8099,7 +8100,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="367" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="367" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A367" t="s">
         <v>523</v>
       </c>
@@ -8113,7 +8114,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="368" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="368" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A368" t="s">
         <v>523</v>
       </c>
@@ -8127,7 +8128,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="369" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="369" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A369" t="s">
         <v>523</v>
       </c>
@@ -8141,7 +8142,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="370" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="370" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A370" t="s">
         <v>523</v>
       </c>
@@ -8155,7 +8156,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="371" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="371" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A371" t="s">
         <v>523</v>
       </c>
@@ -8169,7 +8170,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="372" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="372" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A372" t="s">
         <v>523</v>
       </c>
@@ -8183,7 +8184,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="373" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="373" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A373" t="s">
         <v>523</v>
       </c>
@@ -8197,7 +8198,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="374" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="374" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A374" t="s">
         <v>523</v>
       </c>
@@ -8211,7 +8212,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="375" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="375" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A375" t="s">
         <v>523</v>
       </c>
@@ -8225,7 +8226,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="376" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="376" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A376" t="s">
         <v>523</v>
       </c>
@@ -8239,7 +8240,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="377" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="377" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A377" t="s">
         <v>523</v>
       </c>
@@ -8253,7 +8254,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="378" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="378" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A378" t="s">
         <v>523</v>
       </c>
@@ -8267,7 +8268,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="379" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="379" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A379" t="s">
         <v>523</v>
       </c>
@@ -8281,7 +8282,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="380" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="380" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A380" t="s">
         <v>523</v>
       </c>
@@ -8295,7 +8296,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="381" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="381" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A381" t="s">
         <v>523</v>
       </c>
@@ -8309,7 +8310,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="382" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="382" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A382" t="s">
         <v>523</v>
       </c>
@@ -8323,7 +8324,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="383" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="383" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A383" t="s">
         <v>523</v>
       </c>
@@ -8337,7 +8338,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="384" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="384" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A384" t="s">
         <v>523</v>
       </c>
@@ -8351,7 +8352,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="385" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="385" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A385" t="s">
         <v>523</v>
       </c>
@@ -8365,7 +8366,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="386" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="386" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A386" t="s">
         <v>523</v>
       </c>
@@ -8379,7 +8380,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="387" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="387" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A387" t="s">
         <v>523</v>
       </c>
@@ -8393,7 +8394,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="388" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="388" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A388" t="s">
         <v>523</v>
       </c>
@@ -8407,7 +8408,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="389" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="389" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A389" t="s">
         <v>523</v>
       </c>
@@ -8421,7 +8422,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="390" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="390" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A390" t="s">
         <v>523</v>
       </c>
@@ -8435,7 +8436,7 @@
         <v>545</v>
       </c>
     </row>
-    <row r="391" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="391" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A391" t="s">
         <v>523</v>
       </c>
@@ -8449,7 +8450,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="392" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="392" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A392" t="s">
         <v>523</v>
       </c>
@@ -8463,7 +8464,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="393" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="393" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A393" t="s">
         <v>523</v>
       </c>
@@ -8477,7 +8478,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="394" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="394" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A394" t="s">
         <v>523</v>
       </c>
@@ -8491,7 +8492,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="395" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="395" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A395" t="s">
         <v>523</v>
       </c>
@@ -8505,7 +8506,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="396" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="396" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A396" t="s">
         <v>523</v>
       </c>
@@ -8519,7 +8520,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="397" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="397" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A397" t="s">
         <v>523</v>
       </c>
@@ -8533,7 +8534,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="398" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="398" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A398" t="s">
         <v>523</v>
       </c>
@@ -8547,7 +8548,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="399" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="399" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A399" t="s">
         <v>523</v>
       </c>
@@ -8561,7 +8562,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="400" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="400" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A400" t="s">
         <v>523</v>
       </c>
@@ -8575,7 +8576,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="401" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="401" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A401" t="s">
         <v>523</v>
       </c>
@@ -8589,7 +8590,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="402" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="402" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A402" t="s">
         <v>523</v>
       </c>
@@ -8603,7 +8604,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="403" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="403" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A403" t="s">
         <v>523</v>
       </c>
@@ -8617,7 +8618,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="404" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="404" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A404" t="s">
         <v>523</v>
       </c>
@@ -8631,7 +8632,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="405" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="405" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A405" t="s">
         <v>523</v>
       </c>
@@ -8645,7 +8646,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="406" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="406" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A406" t="s">
         <v>523</v>
       </c>
@@ -8659,7 +8660,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="407" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="407" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A407" t="s">
         <v>523</v>
       </c>
@@ -8673,7 +8674,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="408" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="408" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A408" t="s">
         <v>523</v>
       </c>
@@ -8687,7 +8688,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="409" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="409" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A409" t="s">
         <v>523</v>
       </c>
@@ -8701,7 +8702,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="410" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="410" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A410" t="s">
         <v>523</v>
       </c>
@@ -8715,7 +8716,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="411" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="411" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A411" t="s">
         <v>523</v>
       </c>
@@ -8729,7 +8730,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="412" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="412" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A412" t="s">
         <v>523</v>
       </c>
@@ -8743,7 +8744,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="413" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="413" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A413" t="s">
         <v>523</v>
       </c>
@@ -8757,7 +8758,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="414" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="414" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A414" t="s">
         <v>523</v>
       </c>
@@ -8771,7 +8772,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="415" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="415" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A415" t="s">
         <v>523</v>
       </c>
@@ -8785,7 +8786,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="416" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="416" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A416" t="s">
         <v>523</v>
       </c>
@@ -8799,7 +8800,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="417" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="417" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A417" t="s">
         <v>523</v>
       </c>
@@ -8813,7 +8814,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="418" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="418" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A418" t="s">
         <v>523</v>
       </c>
@@ -8827,7 +8828,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="419" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="419" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A419" t="s">
         <v>523</v>
       </c>
@@ -8841,7 +8842,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="420" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="420" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A420" t="s">
         <v>523</v>
       </c>
@@ -8855,7 +8856,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="421" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="421" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A421" t="s">
         <v>523</v>
       </c>
@@ -8869,7 +8870,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="422" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="422" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A422" t="s">
         <v>523</v>
       </c>
@@ -8883,7 +8884,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="423" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="423" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A423" t="s">
         <v>523</v>
       </c>
@@ -8897,7 +8898,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="424" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="424" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A424" t="s">
         <v>523</v>
       </c>
@@ -8911,7 +8912,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="425" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="425" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A425" t="s">
         <v>523</v>
       </c>
@@ -8925,7 +8926,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="426" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="426" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A426" t="s">
         <v>523</v>
       </c>
@@ -8939,7 +8940,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="427" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="427" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A427" t="s">
         <v>523</v>
       </c>
@@ -8953,7 +8954,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="428" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="428" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A428" t="s">
         <v>523</v>
       </c>
@@ -8967,7 +8968,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="429" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="429" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A429" t="s">
         <v>523</v>
       </c>
@@ -8981,7 +8982,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="430" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="430" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A430" t="s">
         <v>523</v>
       </c>
@@ -8995,7 +8996,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="431" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="431" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A431" t="s">
         <v>523</v>
       </c>
@@ -9009,7 +9010,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="432" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="432" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A432" t="s">
         <v>523</v>
       </c>
@@ -9023,7 +9024,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="433" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="433" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A433" t="s">
         <v>523</v>
       </c>
@@ -9037,7 +9038,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="434" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="434" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A434" t="s">
         <v>523</v>
       </c>
@@ -9051,7 +9052,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="435" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="435" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A435" t="s">
         <v>523</v>
       </c>
@@ -9065,7 +9066,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="436" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="436" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A436" t="s">
         <v>523</v>
       </c>
@@ -9079,7 +9080,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="437" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="437" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A437" t="s">
         <v>523</v>
       </c>
@@ -9093,7 +9094,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="438" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="438" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A438" t="s">
         <v>523</v>
       </c>
@@ -9108,7 +9109,14 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E312" xr:uid="{4F478A83-309B-482A-B8B0-EA389326FD99}"/>
+  <autoFilter ref="A1:E438" xr:uid="{4F478A83-309B-482A-B8B0-EA389326FD99}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="موقع النخيل والزيتون"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>